<commit_message>
fix: correct typo in registration test scenario
</commit_message>
<xml_diff>
--- a/testcases.xlsx
+++ b/testcases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026\Tester\Mini-Booking-Web-App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{113A1C82-BD86-43E0-8EB7-1731ADA5A5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AFEA4E9-75CF-4722-BF08-96F98DEFA390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3A6CB79A-4433-4652-A23D-CF9D73344B39}"/>
+    <workbookView xWindow="9960" yWindow="0" windowWidth="18945" windowHeight="16305" xr2:uid="{3A6CB79A-4433-4652-A23D-CF9D73344B39}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -56,27 +56,44 @@
     <t>Expected Result</t>
   </si>
   <si>
-    <t xml:space="preserve">TC_LOGIN_05_01 </t>
-  </si>
-  <si>
-    <t>TS_LOGIN_05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify user can login with valid credentials  </t>
-  </si>
-  <si>
-    <t>User đã đăng ký tài khoản hợp lệ</t>
-  </si>
-  <si>
-    <t>1. Truy cập trang login
-2. Nhập email: test@gmail.com
-3. Nhập password: 123456
-4. Click nút Login</t>
-  </si>
-  <si>
-    <t>- Hệ thống đăng nhập thành công
-- Chuyển hướng về trang chủ
-- Token được lưu (localStorage/cookie)</t>
+    <t xml:space="preserve">TC_REGISTER_01_01 </t>
+  </si>
+  <si>
+    <t>TS_REGISTER_01</t>
+  </si>
+  <si>
+    <t>Đăng ký khi bỏ trống các trường</t>
+  </si>
+  <si>
+    <t>Không có</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi tại từng field
++ Email: "Email không được để trống"
++ Password: "Password không được để trống"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>- Trình duyệt hiển thị thông báo mặc định "Please fill out this field"
+- Không có message custom từ hệ thống</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Để trống email
+3. Để trống password
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>Note</t>
   </si>
 </sst>
 </file>
@@ -135,13 +152,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -514,53 +534,70 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0232D0E4-DCB2-41A2-A718-3E0DDDCF69F1}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="15.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="70.7109375" style="2" customWidth="1"/>
     <col min="4" max="4" width="50.7109375" style="2" customWidth="1"/>
-    <col min="5" max="6" width="100.7109375" style="2" customWidth="1"/>
+    <col min="5" max="7" width="100.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:9" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>11</v>
+      <c r="E2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update test scenarios and testcases
</commit_message>
<xml_diff>
--- a/testcases.xlsx
+++ b/testcases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026\Tester\Mini-Booking-Web-App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AFEA4E9-75CF-4722-BF08-96F98DEFA390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A34416D-CE09-467F-B3DC-842F275BFAB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9960" yWindow="0" windowWidth="18945" windowHeight="16305" xr2:uid="{3A6CB79A-4433-4652-A23D-CF9D73344B39}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3A6CB79A-4433-4652-A23D-CF9D73344B39}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="69">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -62,9 +62,6 @@
     <t>TS_REGISTER_01</t>
   </si>
   <si>
-    <t>Đăng ký khi bỏ trống các trường</t>
-  </si>
-  <si>
     <t>Không có</t>
   </si>
   <si>
@@ -77,23 +74,234 @@
     <t>FAIL</t>
   </si>
   <si>
-    <t>- Hiển thị message lỗi tại từng field
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Đăng ký khi bỏ trống email</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi 
 + Email: "Email không được để trống"
-+ Password: "Password không được để trống"
 - Không gửi request lên server</t>
   </si>
   <si>
-    <t>- Trình duyệt hiển thị thông báo mặc định "Please fill out this field"
-- Không có message custom từ hệ thống</t>
+    <t>TC_REGISTER_01_02</t>
+  </si>
+  <si>
+    <t>TS_REGISTER_02</t>
+  </si>
+  <si>
+    <t>Đăng ký khi bỏ trống mật khẩu</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi
++ Password: "Mật khẩu không được để trống"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>TC_REGISTER_01_03</t>
+  </si>
+  <si>
+    <t>Đăng ký khi bỏ trống tất cả các trường</t>
   </si>
   <si>
     <t>1. Truy cập trang register
 2. Để trống email
-3. Để trống password
+3. Để trống mật khẩu
 4. Click nút Register</t>
   </si>
   <si>
-    <t>Note</t>
+    <t>- Hiển thị message lỗi
++ Email: "Email không được để trống"
++ Password: "Mật khẩu không được để trống"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>TC_REGISTER_02_01</t>
+  </si>
+  <si>
+    <t>Đăng ký với email sai format</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi
++ Email: "Email không đúng định dạng"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>TC_REGISTER_02_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đăng ký với pasword quá ngắn </t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi 
++ Password: "Password quá ngắn, …yêu cầu thêm"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>TC_REGISTER_02_03</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Nhập email: "test@gmail.com"
+3. Nhập password: "1"
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Nhập email: "testcase02"
+3. Nhập password: "123456"
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Nhập email: "test@gmail.com"
+3. Để trống mật khẩu
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Để trống email
+3. Nhập password: "123456"
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>Đăng ký với email có khoảng trắng ở đầu</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Nhập email: " test@gmail.com"
+3. Nhập password: "1"
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>- Trình duyệt hiển thị thông báo thành công
+- Chuyển hướng về trang login</t>
+  </si>
+  <si>
+    <t>- Đã xử lý khoảng trắng
+- Trình duyệt hiển thị thông báo thành công
+- Chuyển hướng về trang login</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>TC_REGISTER_02_04</t>
+  </si>
+  <si>
+    <t>Đăng ký với email có khoảng trắng ở giữa</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Nhập email: "test @gmail.com"
+3. Nhập password: "1"
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>Đăng ký với email chỉ nhập khoảng trắng</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Nhập email: " "
+3. Nhập password: "1"
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>Đăng ký với password có khoảng trắng ở đầu</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Nhập email: "test@gmail.com"
+3. Nhập password: " 123456"
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>Đăng ký với password có khoảng trắng ở giữa</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Nhập email: "test@gmail.com"
+3. Nhập password: "123 456"
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>Đăng ký với password chỉ nhập khoảng trắng</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Nhập email: "test@gmail.com"
+3. Nhập password: "      "
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t>TC_REGISTER_03_01</t>
+  </si>
+  <si>
+    <t>TS_REGISTER_03</t>
+  </si>
+  <si>
+    <t>Đăng ký với email đã tồn tại</t>
+  </si>
+  <si>
+    <t>Email test@gmail.com đã tồn tại trong hệ thông</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang register
+2. Nhập email: "test@gmail.com"
+3. Nhập password: "123456"
+4. Click nút Register</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Gửi request lên server
+- Hiển thị message lỗi
++ Email: "Email đã tồn tại"
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Có message custom thông báo: "Email already exists"
+- Không tạo tài khoản mới </t>
+  </si>
+  <si>
+    <t>TC_REGISTER_04_01</t>
+  </si>
+  <si>
+    <t>TS_REGISTER_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đăng ký với email hợp lệ và mật khẩu hợp lệ </t>
+  </si>
+  <si>
+    <t>- Gửi request lên server
+- Tạo thành công tài khoản mới</t>
+  </si>
+  <si>
+    <t>- Xử lý khoảng trắng bằng trim()
+- Gửi request lên server
+- Tạo thành công tài khoản mới</t>
+  </si>
+  <si>
+    <t>- Trình duyệt hiển thị validation mặc định, không gửi request
+- Không có message custom từ hệ thống</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Trình duyệt hiển thị validation mặc định, không gửi request
+- Không có message custom từ hệ thống </t>
+  </si>
+  <si>
+    <t>TC_REGISTER_03_02</t>
+  </si>
+  <si>
+    <t>TC_REGISTER_03_03</t>
+  </si>
+  <si>
+    <t>TC_REGISTER_03_04</t>
+  </si>
+  <si>
+    <t>TC_REGISTER_05_01</t>
+  </si>
+  <si>
+    <t>TS_REGISTER_05</t>
   </si>
 </sst>
 </file>
@@ -152,7 +360,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -181,11 +389,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <left style="thin">
@@ -534,7 +763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0232D0E4-DCB2-41A2-A718-3E0DDDCF69F1}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
@@ -565,13 +794,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="I1" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -582,26 +811,338 @@
         <v>7</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>9</v>
-      </c>
       <c r="E2" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>12</v>
+      <c r="B3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:XFD1048576">
+  <conditionalFormatting sqref="A20:XFD1048576 A1:XFD14">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$A1&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
feat: update booking test cases
</commit_message>
<xml_diff>
--- a/testcases.xlsx
+++ b/testcases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026\Tester\Mini-Booking-Web-App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A42FE1-B55D-44B7-BEE5-21C87913C6DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C538AD4-B564-4E98-96D0-A744DC3822AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3A6CB79A-4433-4652-A23D-CF9D73344B39}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{3A6CB79A-4433-4652-A23D-CF9D73344B39}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="209">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -554,6 +554,283 @@
     <t xml:space="preserve">- Có message custom thông báo: "Invalid credentials"
 - Không lưu token
 - Không có hành động chuyển hướng </t>
+  </si>
+  <si>
+    <t>TC_BOOKING_01_01</t>
+  </si>
+  <si>
+    <t>TS_BOOKING_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đặt lịch khi bỏ trống ngày </t>
+  </si>
+  <si>
+    <t>Đặt lịch khi bỏ trống giờ</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_01_02</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_01_03</t>
+  </si>
+  <si>
+    <t>Đặt lịch khi bỏ trống cả ngày và giờ</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_02_01</t>
+  </si>
+  <si>
+    <t>TS_BOOKING_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đặt lịch với ngày của quá khứ </t>
+  </si>
+  <si>
+    <t>TC_BOOKING_02_02</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_02_03</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_03_01</t>
+  </si>
+  <si>
+    <t>TS_BOOKING_03</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_04_01</t>
+  </si>
+  <si>
+    <t>TS_BOOKING_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đặt lịch với ngày hiện tại và giờ hiện tại </t>
+  </si>
+  <si>
+    <t>TC_BOOKING_04_02</t>
+  </si>
+  <si>
+    <t>Đặt lịch với ngày tương lai gần (30 ngày)</t>
+  </si>
+  <si>
+    <t>Đặt lịch với ngày tương lai xa (lớn hơn 30 ngày)</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_04_03</t>
+  </si>
+  <si>
+    <t>Đặt lịch với thời gian tương lai gần (nhỏ hơn 3 tiếng)</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_04_04</t>
+  </si>
+  <si>
+    <t>Đặt lịch với thời gian tương lai xa (lớn hơn 3 tiếng)</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_05_01</t>
+  </si>
+  <si>
+    <t>TS_BOOKING_05</t>
+  </si>
+  <si>
+    <t>Đặt lịch thành công</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_06_01</t>
+  </si>
+  <si>
+    <t>TS_BOOKING_06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xem lịch khi chưa có lịch hẹn </t>
+  </si>
+  <si>
+    <t>Đã đăng nhập</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_06_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xem lịch khi đã có lịch hẹn </t>
+  </si>
+  <si>
+    <t>TC_BOOKING_06_04</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_06_03</t>
+  </si>
+  <si>
+    <t>Chưa đăng nhập</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_02_04</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Để trống ngày
+3. Nhập giờ: "10:33 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_02_05</t>
+  </si>
+  <si>
+    <t>Đặt lịch vào ngày không phục vụ</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_02_06</t>
+  </si>
+  <si>
+    <t>Đặt lịch vào giờ không phục vụ</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_02_07</t>
+  </si>
+  <si>
+    <t>TC_BOOKING_02_09</t>
+  </si>
+  <si>
+    <t>Đặt lịch khi nhập sai format ngày</t>
+  </si>
+  <si>
+    <t>Đặt lịch khi nhập sai format giờ</t>
+  </si>
+  <si>
+    <t>Đặt lịch khi nhập sai format ngày và giờ</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Để trống ngày
+3. Để trống giờ
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>Thời gian hiện tại là ngày 25/03/2026</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "31/03/2026"
+3. Để trống giờ
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "20/03/2026"
+3. Nhập giờ: "10:33 AM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>Đã chọn ngày và thời gian hiện tại là 25/03/2026 13:00 PM</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "31/03/2026"
+3. Nhập giờ: "10:33 AM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đặt lịch với giờ của quá khứ, ngày tương lai </t>
+  </si>
+  <si>
+    <t>Ngày 28/03/2026 không hoạt động</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/03/2026"
+3. Nhập giờ: "10:33 AM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>Đã chọn ngày và sau 10:00 PM không hoạt động</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "31/03/2026"
+3. Nhập giờ: "10:33 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>Đặt lịch vào ngày không phục vụ và giờ không phục vụ</t>
+  </si>
+  <si>
+    <t>Ngày 28/03/2026 không hoạt động và sau 10:00 PM không hoạt động</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/03/2026"
+3. Nhập giờ: "10:33 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "03/28/2026"
+3. Nhập giờ: "10:33 AM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/03/2026"
+3. Nhập giờ: "10h33"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "03/28/2026"
+3. Nhập giờ: "10h33"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>Hiện tại đang là ngày 28/03/2026 và 13:00 PM</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/03/2026"
+3. Nhập giờ: "13:00 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>Hiện tại đang là ngày 28/03/2026</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/04/2026"
+3. Nhập giờ: "13:00 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/05/2026"
+3. Nhập giờ: "13:00 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/03/2026"
+3. Nhập giờ: "14:00 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/03/2026"
+3. Nhập giờ: "19:00 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Truy cập trang booking
+2. Xem danh sách booking ở bên dưới form đặt lịch </t>
+  </si>
+  <si>
+    <t>TC_BOOKING_07_01</t>
+  </si>
+  <si>
+    <t>TS_BOOKING_07</t>
+  </si>
+  <si>
+    <t>Đặt lịch trùng thời gian</t>
+  </si>
+  <si>
+    <t>Đã có lịch tại thời điểm ngày 28/03/2026 và 13:00 PM</t>
   </si>
 </sst>
 </file>
@@ -645,331 +922,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="29">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="11">
     <dxf>
       <border>
         <left style="thin">
@@ -1498,19 +1451,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0232D0E4-DCB2-41A2-A718-3E0DDDCF69F1}">
-  <dimension ref="A1:I31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I53"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="8" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" style="8" customWidth="1"/>
-    <col min="3" max="3" width="70.7109375" style="4" customWidth="1"/>
-    <col min="4" max="4" width="50.7109375" style="4" customWidth="1"/>
-    <col min="5" max="7" width="100.7109375" style="4" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" style="8"/>
-    <col min="9" max="16384" width="9.140625" style="9"/>
+    <col min="1" max="1" width="20.6640625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="70.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="50.6640625" style="4" customWidth="1"/>
+    <col min="5" max="7" width="100.6640625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" style="8"/>
+    <col min="9" max="16384" width="9.109375" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1539,7 +1492,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
@@ -1565,7 +1518,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>15</v>
       </c>
@@ -1591,7 +1544,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>19</v>
       </c>
@@ -1617,7 +1570,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>23</v>
       </c>
@@ -1643,7 +1596,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>26</v>
       </c>
@@ -1669,7 +1622,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>29</v>
       </c>
@@ -1695,7 +1648,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>39</v>
       </c>
@@ -1721,7 +1674,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>50</v>
       </c>
@@ -1747,7 +1700,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>63</v>
       </c>
@@ -1773,7 +1726,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>64</v>
       </c>
@@ -1799,7 +1752,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>65</v>
       </c>
@@ -1825,7 +1778,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>56</v>
       </c>
@@ -1851,7 +1804,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>66</v>
       </c>
@@ -1877,7 +1830,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>68</v>
       </c>
@@ -1903,7 +1856,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>71</v>
       </c>
@@ -1929,7 +1882,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>76</v>
       </c>
@@ -1955,7 +1908,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>81</v>
       </c>
@@ -1981,7 +1934,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>84</v>
       </c>
@@ -2007,7 +1960,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>88</v>
       </c>
@@ -2033,7 +1986,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>91</v>
       </c>
@@ -2059,7 +2012,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>94</v>
       </c>
@@ -2085,7 +2038,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>98</v>
       </c>
@@ -2111,7 +2064,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>101</v>
       </c>
@@ -2137,7 +2090,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>127</v>
       </c>
@@ -2163,7 +2116,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>128</v>
       </c>
@@ -2189,7 +2142,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>104</v>
       </c>
@@ -2215,7 +2168,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>108</v>
       </c>
@@ -2241,7 +2194,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
         <v>112</v>
       </c>
@@ -2267,7 +2220,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
         <v>116</v>
       </c>
@@ -2293,7 +2246,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>118</v>
       </c>
@@ -2319,150 +2272,434 @@
         <v>38</v>
       </c>
     </row>
+    <row r="32" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A39" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A50" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A52" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A53" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:XFD14 C19:C20 C21:E21 C28:C29 C31 C18:F18 A32:XFD1048576 C22:C26 I18:XFD18 C27:G27 C30:G30 E19:XFD19 E20:F20 E31:XFD31 E22:G26 E28:G29 I20:XFD30">
-    <cfRule type="expression" dxfId="28" priority="30">
+  <conditionalFormatting sqref="A18:B31 E32 A32:D37 F32:XFD37 E36:E39 A38:XFD1048576">
+    <cfRule type="expression" dxfId="10" priority="27">
+      <formula>$A18&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A15:F17">
+    <cfRule type="expression" dxfId="9" priority="19">
+      <formula>$A15&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:XFD14 C18:F18 E19:XFD19 E20:F20">
+    <cfRule type="expression" dxfId="8" priority="32">
       <formula>$A1&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A15:E15 I15:XFD15">
-    <cfRule type="expression" dxfId="27" priority="29">
+  <conditionalFormatting sqref="C19:D20">
+    <cfRule type="expression" dxfId="7" priority="26">
+      <formula>$A19&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C21:F21">
+    <cfRule type="expression" dxfId="6" priority="18">
+      <formula>$A21&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C22:G30">
+    <cfRule type="expression" dxfId="5" priority="24">
+      <formula>$A22&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C31:XFD31">
+    <cfRule type="expression" dxfId="4" priority="22">
+      <formula>$A31&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G20:G21">
+    <cfRule type="expression" dxfId="3" priority="13">
+      <formula>$A20&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G15:XFD18">
+    <cfRule type="expression" dxfId="2" priority="15">
       <formula>$A15&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A16:C16 I16:XFD16 E16">
-    <cfRule type="expression" dxfId="26" priority="28">
-      <formula>$A16&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A17:E17 I17:XFD17">
-    <cfRule type="expression" dxfId="25" priority="27">
-      <formula>$A17&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A18:A31">
-    <cfRule type="expression" dxfId="24" priority="26">
-      <formula>$A18&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B18:B31">
-    <cfRule type="expression" dxfId="23" priority="25">
-      <formula>$A18&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D19:D20">
-    <cfRule type="expression" dxfId="22" priority="24">
-      <formula>$A19&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D22:D26">
-    <cfRule type="expression" dxfId="15" priority="23">
-      <formula>$A22&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D28:D29">
-    <cfRule type="expression" dxfId="21" priority="22">
-      <formula>$A28&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D31">
-    <cfRule type="expression" dxfId="20" priority="20">
-      <formula>$A31&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F15">
-    <cfRule type="expression" dxfId="19" priority="19">
-      <formula>$A15&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F16:F17">
-    <cfRule type="expression" dxfId="18" priority="18">
-      <formula>$A16&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D16">
-    <cfRule type="expression" dxfId="17" priority="17">
-      <formula>$A16&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F21">
-    <cfRule type="expression" dxfId="16" priority="16">
-      <formula>$A21&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G15:G18">
-    <cfRule type="expression" dxfId="14" priority="15">
-      <formula>$A15&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H15">
-    <cfRule type="expression" dxfId="13" priority="14">
-      <formula>$A15&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H16:H18">
-    <cfRule type="expression" dxfId="12" priority="13">
-      <formula>$A16&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G21">
-    <cfRule type="expression" dxfId="11" priority="12">
-      <formula>$A21&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G20">
-    <cfRule type="expression" dxfId="10" priority="11">
+  <conditionalFormatting sqref="H20:XFD30">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>$A20&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H20">
-    <cfRule type="expression" dxfId="9" priority="10">
-      <formula>$A20&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H21">
-    <cfRule type="expression" dxfId="8" priority="9">
-      <formula>$A21&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H22">
-    <cfRule type="expression" dxfId="7" priority="8">
-      <formula>$A22&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H23">
-    <cfRule type="expression" dxfId="6" priority="7">
-      <formula>$A23&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H24">
-    <cfRule type="expression" dxfId="5" priority="6">
-      <formula>$A24&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H25">
-    <cfRule type="expression" dxfId="4" priority="5">
-      <formula>$A25&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H26">
-    <cfRule type="expression" dxfId="3" priority="4">
-      <formula>$A26&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H27">
-    <cfRule type="expression" dxfId="2" priority="3">
-      <formula>$A27&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H28">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$A28&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H29:H30">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>$A29&lt;&gt;""</formula>
+  <conditionalFormatting sqref="E33:E35">
+    <cfRule type="expression" dxfId="0" priority="35">
+      <formula>$A33&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: update booking test scenario for time conflict and modify test cases
</commit_message>
<xml_diff>
--- a/testcases.xlsx
+++ b/testcases.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026\Tester\Mini-Booking-Web-App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C538AD4-B564-4E98-96D0-A744DC3822AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6843B1AC-19BE-46A5-A3BB-3641D0021A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{3A6CB79A-4433-4652-A23D-CF9D73344B39}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3A6CB79A-4433-4652-A23D-CF9D73344B39}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="testcase_booking_basic" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="225">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -721,18 +721,12 @@
 4. Click nút Tạo booking</t>
   </si>
   <si>
-    <t>Đã chọn ngày và thời gian hiện tại là 25/03/2026 13:00 PM</t>
-  </si>
-  <si>
     <t>1. Truy cập trang booking
 2. Nhập ngày: "31/03/2026"
 3. Nhập giờ: "10:33 AM"
 4. Click nút Tạo booking</t>
   </si>
   <si>
-    <t xml:space="preserve">Đặt lịch với giờ của quá khứ, ngày tương lai </t>
-  </si>
-  <si>
     <t>Ngày 28/03/2026 không hoạt động</t>
   </si>
   <si>
@@ -781,28 +775,7 @@
 4. Click nút Tạo booking</t>
   </si>
   <si>
-    <t>Hiện tại đang là ngày 28/03/2026 và 13:00 PM</t>
-  </si>
-  <si>
-    <t>1. Truy cập trang booking
-2. Nhập ngày: "28/03/2026"
-3. Nhập giờ: "13:00 PM"
-4. Click nút Tạo booking</t>
-  </si>
-  <si>
     <t>Hiện tại đang là ngày 28/03/2026</t>
-  </si>
-  <si>
-    <t>1. Truy cập trang booking
-2. Nhập ngày: "28/04/2026"
-3. Nhập giờ: "13:00 PM"
-4. Click nút Tạo booking</t>
-  </si>
-  <si>
-    <t>1. Truy cập trang booking
-2. Nhập ngày: "28/05/2026"
-3. Nhập giờ: "13:00 PM"
-4. Click nút Tạo booking</t>
   </si>
   <si>
     <t>1. Truy cập trang booking
@@ -830,7 +803,111 @@
     <t>Đặt lịch trùng thời gian</t>
   </si>
   <si>
-    <t>Đã có lịch tại thời điểm ngày 28/03/2026 và 13:00 PM</t>
+    <t>- Hiển thị message lỗi
++ "Không được để trống ngày"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi
++ "Không được để trống giờ"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi
++ "Không được để trống ngày"
++ "Không được để trống giờ"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi
++ "Không được đặt ngày ở quá khứ"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>- Gửi request lên server
+- Đặt lịch thành công</t>
+  </si>
+  <si>
+    <t>- Gửi request lên server
+- Server phản hồi không thể đặt được lịch thời gian này cùng với lý do</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi
++ "Ngày không đúng định dạng"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi
++ "Giờ không đúng định dạng"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi
++ "Ngày  không đúng định dạng"
++ "Giờ  không đúng định dạng"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi
++ "Không thể đặt lịch trong phạm vi 30 ngày tính từ hiện tại"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>- Hiển thị message lỗi
++ "Không thể đặt lịch trong phạm vi 3 tiếng tính từ hiện tại"
+- Không gửi request lên server</t>
+  </si>
+  <si>
+    <t>- Gửi request lên server
+- Nhận response và hiển thị lên màn hình</t>
+  </si>
+  <si>
+    <t>- Gửi request lên server
+- Nhận response và hiển thị lên màn hình, có chú thích khi chưa có lịch</t>
+  </si>
+  <si>
+    <t>- Gửi request lên server
+- Nhận response và hiển thị lên màn hình
+- Không có chú thích nếu lịch trống</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Không gửi request lên server
+- Yêu cầu đăng nhập</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Gửi request lên server
+- Báo lỗi đặt lịch trùng thời gian
+</t>
+  </si>
+  <si>
+    <t>Thời gian hiện tại là 25/03/2026 01:00 PM</t>
+  </si>
+  <si>
+    <t>Hiện tại đang là ngày 28/03/2026 và 01:00 PM</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/03/2026"
+3. Nhập giờ: "01:00 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/04/2026"
+3. Nhập giờ: "01:00 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang booking
+2. Nhập ngày: "28/05/2026"
+3. Nhập giờ: "01:00 PM"
+4. Click nút Tạo booking</t>
+  </si>
+  <si>
+    <t>Đã có lịch tại thời điểm ngày 28/03/2026 và 01:00 PM</t>
+  </si>
+  <si>
+    <t>Đặt lịch với ngày tương lai và giờ nhỏ hơn hiện tại</t>
   </si>
 </sst>
 </file>
@@ -922,7 +999,223 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="23">
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <left style="thin">
@@ -1452,18 +1745,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0232D0E4-DCB2-41A2-A718-3E0DDDCF69F1}">
   <dimension ref="A1:I53"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" style="8" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="70.6640625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="50.6640625" style="4" customWidth="1"/>
-    <col min="5" max="7" width="100.6640625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" style="8"/>
-    <col min="9" max="16384" width="9.109375" style="9"/>
+    <col min="1" max="1" width="20.7109375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="70.7109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="50.7109375" style="4" customWidth="1"/>
+    <col min="5" max="7" width="100.7109375" style="4" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="8"/>
+    <col min="9" max="16384" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1492,7 +1785,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
@@ -1518,7 +1811,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>15</v>
       </c>
@@ -1544,7 +1837,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>19</v>
       </c>
@@ -1570,7 +1863,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>23</v>
       </c>
@@ -1596,7 +1889,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>26</v>
       </c>
@@ -1622,7 +1915,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>29</v>
       </c>
@@ -1648,7 +1941,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>39</v>
       </c>
@@ -1674,7 +1967,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>50</v>
       </c>
@@ -1700,7 +1993,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>63</v>
       </c>
@@ -1726,7 +2019,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>64</v>
       </c>
@@ -1752,7 +2045,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>65</v>
       </c>
@@ -1778,7 +2071,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>56</v>
       </c>
@@ -1804,7 +2097,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>66</v>
       </c>
@@ -1830,7 +2123,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>68</v>
       </c>
@@ -1856,7 +2149,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>71</v>
       </c>
@@ -1882,7 +2175,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>76</v>
       </c>
@@ -1908,7 +2201,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>81</v>
       </c>
@@ -1934,7 +2227,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>84</v>
       </c>
@@ -1960,7 +2253,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>88</v>
       </c>
@@ -1986,7 +2279,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>91</v>
       </c>
@@ -2012,7 +2305,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>94</v>
       </c>
@@ -2038,7 +2331,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>98</v>
       </c>
@@ -2064,7 +2357,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>101</v>
       </c>
@@ -2090,7 +2383,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>127</v>
       </c>
@@ -2116,7 +2409,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>128</v>
       </c>
@@ -2142,7 +2435,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>104</v>
       </c>
@@ -2168,7 +2461,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>108</v>
       </c>
@@ -2194,7 +2487,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>112</v>
       </c>
@@ -2220,7 +2513,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>116</v>
       </c>
@@ -2246,7 +2539,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>118</v>
       </c>
@@ -2272,7 +2565,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>133</v>
       </c>
@@ -2288,8 +2581,17 @@
       <c r="E32" s="4" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F32" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H32" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
         <v>137</v>
       </c>
@@ -2305,8 +2607,17 @@
       <c r="E33" s="4" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F33" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H33" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>138</v>
       </c>
@@ -2322,8 +2633,17 @@
       <c r="E34" s="4" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F34" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H34" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>140</v>
       </c>
@@ -2339,8 +2659,17 @@
       <c r="E35" s="4" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F35" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H35" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
         <v>143</v>
       </c>
@@ -2348,16 +2677,25 @@
         <v>141</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>186</v>
+        <v>224</v>
       </c>
       <c r="D36" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E36" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="E36" s="4" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F36" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H36" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
         <v>144</v>
       </c>
@@ -2368,13 +2706,22 @@
         <v>172</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>186</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H37" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
         <v>169</v>
       </c>
@@ -2385,13 +2732,22 @@
         <v>174</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>188</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
         <v>171</v>
       </c>
@@ -2399,16 +2755,25 @@
         <v>141</v>
       </c>
       <c r="C39" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D39" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F39" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H39" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>173</v>
       </c>
@@ -2422,10 +2787,19 @@
         <v>8</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>192</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H40" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
         <v>175</v>
       </c>
@@ -2439,10 +2813,19 @@
         <v>8</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H41" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
         <v>176</v>
       </c>
@@ -2456,10 +2839,19 @@
         <v>8</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>194</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H42" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
         <v>145</v>
       </c>
@@ -2470,13 +2862,22 @@
         <v>149</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>197</v>
+        <v>219</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>220</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H43" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
         <v>147</v>
       </c>
@@ -2487,13 +2888,22 @@
         <v>151</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>221</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H44" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
         <v>150</v>
       </c>
@@ -2504,13 +2914,22 @@
         <v>152</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>222</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H45" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
         <v>153</v>
       </c>
@@ -2521,13 +2940,22 @@
         <v>154</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>197</v>
+        <v>219</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>196</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H46" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
         <v>155</v>
       </c>
@@ -2538,13 +2966,22 @@
         <v>156</v>
       </c>
       <c r="D47" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="E47" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="E47" s="4" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F47" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H47" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
         <v>157</v>
       </c>
@@ -2558,10 +2995,19 @@
         <v>8</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>197</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H48" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
         <v>160</v>
       </c>
@@ -2575,10 +3021,19 @@
         <v>163</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="H49" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
         <v>164</v>
       </c>
@@ -2592,10 +3047,19 @@
         <v>163</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="H50" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
         <v>167</v>
       </c>
@@ -2609,10 +3073,19 @@
         <v>168</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H51" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
         <v>166</v>
       </c>
@@ -2626,80 +3099,158 @@
         <v>168</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H52" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B53" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="G53" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="C53" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>198</v>
+      <c r="H53" s="8" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A18:B31 E32 A32:D37 F32:XFD37 E36:E39 A38:XFD1048576">
-    <cfRule type="expression" dxfId="10" priority="27">
+  <conditionalFormatting sqref="A18:B31 A32:D37 E32:E39 F32:F35 I32:XFD35 H36:XFD36 F37:F43 A38:F43 I37:XFD43 A44:E44 H44:XFD44 A45:F46 I45:XFD46 A47:E48 H47:XFD48 A49:G49 I49:XFD49 A50:XFD52 A54:XFD1048576 A53:F53 I53:XFD53">
+    <cfRule type="expression" dxfId="22" priority="40">
       <formula>$A18&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A15:F17">
-    <cfRule type="expression" dxfId="9" priority="19">
+    <cfRule type="expression" dxfId="21" priority="32">
       <formula>$A15&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:XFD14 C18:F18 E19:XFD19 E20:F20">
-    <cfRule type="expression" dxfId="8" priority="32">
+    <cfRule type="expression" dxfId="20" priority="45">
       <formula>$A1&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19:D20">
-    <cfRule type="expression" dxfId="7" priority="26">
+    <cfRule type="expression" dxfId="19" priority="39">
       <formula>$A19&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C21:F21">
-    <cfRule type="expression" dxfId="6" priority="18">
+    <cfRule type="expression" dxfId="18" priority="31">
       <formula>$A21&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C22:G30">
-    <cfRule type="expression" dxfId="5" priority="24">
+    <cfRule type="expression" dxfId="17" priority="37">
       <formula>$A22&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C31:XFD31">
-    <cfRule type="expression" dxfId="4" priority="22">
+    <cfRule type="expression" dxfId="16" priority="35">
       <formula>$A31&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G20:G21">
-    <cfRule type="expression" dxfId="3" priority="13">
+    <cfRule type="expression" dxfId="15" priority="26">
       <formula>$A20&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G15:XFD18">
-    <cfRule type="expression" dxfId="2" priority="15">
+    <cfRule type="expression" dxfId="14" priority="28">
       <formula>$A15&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H20:XFD30">
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="13" priority="16">
       <formula>$A20&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E33:E35">
-    <cfRule type="expression" dxfId="0" priority="35">
-      <formula>$A33&lt;&gt;""</formula>
+  <conditionalFormatting sqref="G32:G35">
+    <cfRule type="expression" dxfId="12" priority="13">
+      <formula>$A32&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H32:H35">
+    <cfRule type="expression" dxfId="11" priority="12">
+      <formula>$A32&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F36:G36">
+    <cfRule type="expression" dxfId="10" priority="11">
+      <formula>$A36&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G37:G39">
+    <cfRule type="expression" dxfId="9" priority="10">
+      <formula>$A37&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37:H43">
+    <cfRule type="expression" dxfId="8" priority="9">
+      <formula>$A37&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G40:G42">
+    <cfRule type="expression" dxfId="7" priority="8">
+      <formula>$A40&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G43:G48">
+    <cfRule type="expression" dxfId="6" priority="7">
+      <formula>$A43&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F44">
+    <cfRule type="expression" dxfId="5" priority="6">
+      <formula>$A44&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H45:H46">
+    <cfRule type="expression" dxfId="4" priority="5">
+      <formula>$A45&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F47:F48">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>$A47&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H49">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>$A49&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G53">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$A53&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H53">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$A53&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>